<commit_message>
53 Cf Jobtype change
</commit_message>
<xml_diff>
--- a/TestData/LV_TMTT0046653_VerifyTailExpireFieldOnCFEngagementwithJobTypeShowsValidationWhileChangingStage.xlsx
+++ b/TestData/LV_TMTT0046653_VerifyTailExpireFieldOnCFEngagementwithJobTypeShowsValidationWhileChangingStage.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vkumar0427\source\repos\SF_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32EB542F-067E-45D7-AEB0-175C3E385282}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D199CD98-9B50-4E59-AA5B-08B5203996EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23148" yWindow="708" windowWidth="23256" windowHeight="12456" tabRatio="548" firstSheet="2" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-25044" yWindow="1248" windowWidth="21600" windowHeight="11160" tabRatio="548" firstSheet="2" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="StandardUsers" sheetId="2" r:id="rId1"/>
@@ -291,7 +291,7 @@
     <t>Went To Market?OutcomeTail ExpiresPreparation Effort</t>
   </si>
   <si>
-    <t>Debt Capital Markets</t>
+    <t>Debt Financing</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Tail expires and 69
</commit_message>
<xml_diff>
--- a/TestData/LV_TMTT0046653_VerifyTailExpireFieldOnCFEngagementwithJobTypeShowsValidationWhileChangingStage.xlsx
+++ b/TestData/LV_TMTT0046653_VerifyTailExpireFieldOnCFEngagementwithJobTypeShowsValidationWhileChangingStage.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vkumar0427\source\repos\SF_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{306582F4-0A0A-439D-BAC4-C562D90D3D86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B769D7FD-0217-4950-9640-DC61EED6C42E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="548" firstSheet="2" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-23148" yWindow="708" windowWidth="23256" windowHeight="12456" tabRatio="548" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="StandardUsers" sheetId="2" r:id="rId1"/>
@@ -264,9 +264,6 @@
     <t>Engagements</t>
   </si>
   <si>
-    <t>Jennie Stewart</t>
-  </si>
-  <si>
     <t>Hold</t>
   </si>
   <si>
@@ -295,6 +292,9 @@
   </si>
   <si>
     <t>Verbally Engaged</t>
+  </si>
+  <si>
+    <t>Brian Miller</t>
   </si>
 </sst>
 </file>
@@ -1059,7 +1059,7 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>73</v>
+        <v>83</v>
       </c>
       <c r="B2" t="s">
         <v>9</v>
@@ -1067,10 +1067,10 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>76</v>
+      </c>
+      <c r="B3" t="s">
         <v>77</v>
-      </c>
-      <c r="B3" t="s">
-        <v>78</v>
       </c>
     </row>
   </sheetData>
@@ -1426,7 +1426,7 @@
         <v>39</v>
       </c>
       <c r="C4" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D4" t="s">
         <v>71</v>
@@ -1599,22 +1599,22 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
   </sheetData>
@@ -1632,17 +1632,17 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
   </sheetData>

</xml_diff>